<commit_message>
Issue report 1.0.15: comment Excel font, column order, no filters
- Comment workbooks use the Hyundai Sans Text Medium font (same as the
  post list) instead of Helvetica Neue / Batang
- Columns: domain, text, written date, post URL, then sentiment as the
  rightmost column (title merged across, sentiment colors follow it)
- The raw comment file has no sentiment column; only the sentiment
  analysis file has it
- No auto-filter on comment workbooks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WpiCm7gjqZEZ89dLNZrKh1
</commit_message>
<xml_diff>
--- a/issue-report-extension/templates/comments-template.xlsx
+++ b/issue-report-extension/templates/comments-template.xlsx
@@ -20,18 +20,18 @@
     <font>
       <sz val="10"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
+      <name val="현대산스 Text Medium"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
+      <name val="현대산스 Text Medium"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="나눔명조"/>
+      <name val="현대산스 Text Medium"/>
       <family val="3"/>
       <charset val="129"/>
     </font>
@@ -39,27 +39,27 @@
       <b/>
       <sz val="16"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
+      <name val="현대산스 Text Medium"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <name val="Batang"/>
+      <name val="현대산스 Text Medium"/>
       <family val="2"/>
       <charset val="129"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <name val="Batang"/>
+      <name val="현대산스 Text Medium"/>
       <family val="1"/>
       <charset val="129"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <name val="Helvetica Neue"/>
+      <name val="현대산스 Text Medium"/>
       <family val="2"/>
     </font>
   </fonts>

</xml_diff>